<commit_message>
Sprint 2 CI-005 website composition complete
</commit_message>
<xml_diff>
--- a/output/ClubHubInsight.xlsx
+++ b/output/ClubHubInsight.xlsx
@@ -80,13 +80,13 @@
     <t>Crawl Date</t>
   </si>
   <si>
-    <t>02/09/2026, 00:11:04</t>
+    <t>02/09/2026, 00:36:22</t>
   </si>
   <si>
     <t>Crawl Duration</t>
   </si>
   <si>
-    <t>4m 45s</t>
+    <t>4m 39s</t>
   </si>
   <si>
     <t>Version</t>
@@ -137,7 +137,7 @@
     <t>Average Page Load (ms)</t>
   </si>
   <si>
-    <t>5516 ms</t>
+    <t>5422 ms</t>
   </si>
   <si>
     <t>Site Structure</t>
@@ -3258,7 +3258,7 @@
         <v>121</v>
       </c>
       <c r="T2" s="22">
-        <v>4977</v>
+        <v>4059</v>
       </c>
       <c r="U2" s="19" t="s">
         <v>122</v>
@@ -3329,7 +3329,7 @@
         <v>130</v>
       </c>
       <c r="T3" s="22">
-        <v>4184</v>
+        <v>4003</v>
       </c>
       <c r="U3" s="19" t="s">
         <v>122</v>
@@ -3400,7 +3400,7 @@
         <v>13</v>
       </c>
       <c r="T4" s="22">
-        <v>5443</v>
+        <v>5870</v>
       </c>
       <c r="U4" s="25" t="s">
         <v>135</v>
@@ -3471,7 +3471,7 @@
         <v>13</v>
       </c>
       <c r="T5" s="22">
-        <v>5413</v>
+        <v>5362</v>
       </c>
       <c r="U5" s="25" t="s">
         <v>135</v>
@@ -3542,7 +3542,7 @@
         <v>13</v>
       </c>
       <c r="T6" s="22">
-        <v>5497</v>
+        <v>5682</v>
       </c>
       <c r="U6" s="25" t="s">
         <v>135</v>
@@ -3613,7 +3613,7 @@
         <v>13</v>
       </c>
       <c r="T7" s="22">
-        <v>4576</v>
+        <v>4664</v>
       </c>
       <c r="U7" s="25" t="s">
         <v>135</v>
@@ -3684,7 +3684,7 @@
         <v>13</v>
       </c>
       <c r="T8" s="22">
-        <v>5095</v>
+        <v>4303</v>
       </c>
       <c r="U8" s="25" t="s">
         <v>135</v>
@@ -3755,7 +3755,7 @@
         <v>13</v>
       </c>
       <c r="T9" s="22">
-        <v>4389</v>
+        <v>4702</v>
       </c>
       <c r="U9" s="25" t="s">
         <v>135</v>
@@ -3826,7 +3826,7 @@
         <v>13</v>
       </c>
       <c r="T10" s="22">
-        <v>5218</v>
+        <v>5212</v>
       </c>
       <c r="U10" s="25" t="s">
         <v>135</v>
@@ -3897,7 +3897,7 @@
         <v>13</v>
       </c>
       <c r="T11" s="22">
-        <v>4845</v>
+        <v>5280</v>
       </c>
       <c r="U11" s="25" t="s">
         <v>135</v>
@@ -3968,7 +3968,7 @@
         <v>160</v>
       </c>
       <c r="T12" s="22">
-        <v>4284</v>
+        <v>4719</v>
       </c>
       <c r="U12" s="19" t="s">
         <v>122</v>
@@ -4039,7 +4039,7 @@
         <v>13</v>
       </c>
       <c r="T13" s="22">
-        <v>4893</v>
+        <v>4092</v>
       </c>
       <c r="U13" s="25" t="s">
         <v>135</v>
@@ -4110,7 +4110,7 @@
         <v>13</v>
       </c>
       <c r="T14" s="22">
-        <v>6146</v>
+        <v>5277</v>
       </c>
       <c r="U14" s="25" t="s">
         <v>135</v>
@@ -4181,7 +4181,7 @@
         <v>168</v>
       </c>
       <c r="T15" s="22">
-        <v>4806</v>
+        <v>4939</v>
       </c>
       <c r="U15" s="19" t="s">
         <v>122</v>
@@ -4252,7 +4252,7 @@
         <v>13</v>
       </c>
       <c r="T16" s="22">
-        <v>4828</v>
+        <v>5978</v>
       </c>
       <c r="U16" s="25" t="s">
         <v>135</v>
@@ -4323,7 +4323,7 @@
         <v>13</v>
       </c>
       <c r="T17" s="22">
-        <v>5263</v>
+        <v>4866</v>
       </c>
       <c r="U17" s="25" t="s">
         <v>135</v>
@@ -4394,7 +4394,7 @@
         <v>13</v>
       </c>
       <c r="T18" s="22">
-        <v>5545</v>
+        <v>5417</v>
       </c>
       <c r="U18" s="25" t="s">
         <v>135</v>
@@ -4465,7 +4465,7 @@
         <v>13</v>
       </c>
       <c r="T19" s="22">
-        <v>5338</v>
+        <v>5441</v>
       </c>
       <c r="U19" s="25" t="s">
         <v>135</v>
@@ -4536,7 +4536,7 @@
         <v>13</v>
       </c>
       <c r="T20" s="22">
-        <v>5939</v>
+        <v>4953</v>
       </c>
       <c r="U20" s="25" t="s">
         <v>135</v>
@@ -4607,7 +4607,7 @@
         <v>13</v>
       </c>
       <c r="T21" s="22">
-        <v>4286</v>
+        <v>3836</v>
       </c>
       <c r="U21" s="25" t="s">
         <v>135</v>
@@ -4678,7 +4678,7 @@
         <v>13</v>
       </c>
       <c r="T22" s="22">
-        <v>5003</v>
+        <v>5569</v>
       </c>
       <c r="U22" s="25" t="s">
         <v>135</v>
@@ -4749,7 +4749,7 @@
         <v>13</v>
       </c>
       <c r="T23" s="22">
-        <v>4653</v>
+        <v>4554</v>
       </c>
       <c r="U23" s="25" t="s">
         <v>135</v>
@@ -4820,7 +4820,7 @@
         <v>13</v>
       </c>
       <c r="T24" s="22">
-        <v>5184</v>
+        <v>4854</v>
       </c>
       <c r="U24" s="25" t="s">
         <v>135</v>
@@ -4891,7 +4891,7 @@
         <v>13</v>
       </c>
       <c r="T25" s="22">
-        <v>4890</v>
+        <v>5357</v>
       </c>
       <c r="U25" s="25" t="s">
         <v>135</v>
@@ -4962,7 +4962,7 @@
         <v>13</v>
       </c>
       <c r="T26" s="22">
-        <v>5358</v>
+        <v>5179</v>
       </c>
       <c r="U26" s="25" t="s">
         <v>135</v>
@@ -5033,7 +5033,7 @@
         <v>13</v>
       </c>
       <c r="T27" s="22">
-        <v>4796</v>
+        <v>4988</v>
       </c>
       <c r="U27" s="25" t="s">
         <v>135</v>
@@ -5104,7 +5104,7 @@
         <v>13</v>
       </c>
       <c r="T28" s="22">
-        <v>4114</v>
+        <v>4653</v>
       </c>
       <c r="U28" s="25" t="s">
         <v>135</v>
@@ -5175,7 +5175,7 @@
         <v>200</v>
       </c>
       <c r="T29" s="22">
-        <v>4919</v>
+        <v>4242</v>
       </c>
       <c r="U29" s="19" t="s">
         <v>122</v>
@@ -5246,7 +5246,7 @@
         <v>13</v>
       </c>
       <c r="T30" s="22">
-        <v>5341</v>
+        <v>5270</v>
       </c>
       <c r="U30" s="25" t="s">
         <v>135</v>
@@ -5317,7 +5317,7 @@
         <v>13</v>
       </c>
       <c r="T31" s="22">
-        <v>5399</v>
+        <v>4931</v>
       </c>
       <c r="U31" s="25" t="s">
         <v>135</v>
@@ -5388,7 +5388,7 @@
         <v>13</v>
       </c>
       <c r="T32" s="22">
-        <v>6548</v>
+        <v>4343</v>
       </c>
       <c r="U32" s="25" t="s">
         <v>135</v>
@@ -5459,7 +5459,7 @@
         <v>13</v>
       </c>
       <c r="T33" s="22">
-        <v>5924</v>
+        <v>5505</v>
       </c>
       <c r="U33" s="25" t="s">
         <v>135</v>
@@ -5530,7 +5530,7 @@
         <v>13</v>
       </c>
       <c r="T34" s="22">
-        <v>5184</v>
+        <v>5367</v>
       </c>
       <c r="U34" s="25" t="s">
         <v>135</v>
@@ -5601,7 +5601,7 @@
         <v>13</v>
       </c>
       <c r="T35" s="22">
-        <v>5033</v>
+        <v>5118</v>
       </c>
       <c r="U35" s="25" t="s">
         <v>135</v>
@@ -5672,7 +5672,7 @@
         <v>13</v>
       </c>
       <c r="T36" s="22">
-        <v>4226</v>
+        <v>4056</v>
       </c>
       <c r="U36" s="25" t="s">
         <v>135</v>
@@ -5743,7 +5743,7 @@
         <v>13</v>
       </c>
       <c r="T37" s="22">
-        <v>5371</v>
+        <v>5277</v>
       </c>
       <c r="U37" s="25" t="s">
         <v>135</v>
@@ -5812,7 +5812,7 @@
         <v>13</v>
       </c>
       <c r="T38" s="22">
-        <v>30132</v>
+        <v>30120</v>
       </c>
       <c r="U38" s="25" t="s">
         <v>135</v>
@@ -5883,7 +5883,7 @@
         <v>13</v>
       </c>
       <c r="T39" s="22">
-        <v>6727</v>
+        <v>5059</v>
       </c>
       <c r="U39" s="25" t="s">
         <v>135</v>
@@ -5954,7 +5954,7 @@
         <v>225</v>
       </c>
       <c r="T40" s="22">
-        <v>4380</v>
+        <v>4059</v>
       </c>
       <c r="U40" s="19" t="s">
         <v>122</v>
@@ -6025,7 +6025,7 @@
         <v>229</v>
       </c>
       <c r="T41" s="22">
-        <v>4780</v>
+        <v>4685</v>
       </c>
       <c r="U41" s="19" t="s">
         <v>122</v>
@@ -6096,7 +6096,7 @@
         <v>234</v>
       </c>
       <c r="T42" s="22">
-        <v>4776</v>
+        <v>4863</v>
       </c>
       <c r="U42" s="19" t="s">
         <v>122</v>
@@ -6167,7 +6167,7 @@
         <v>238</v>
       </c>
       <c r="T43" s="22">
-        <v>4108</v>
+        <v>4315</v>
       </c>
       <c r="U43" s="19" t="s">
         <v>122</v>
@@ -6238,7 +6238,7 @@
         <v>242</v>
       </c>
       <c r="T44" s="22">
-        <v>4239</v>
+        <v>4210</v>
       </c>
       <c r="U44" s="19" t="s">
         <v>122</v>
@@ -6309,7 +6309,7 @@
         <v>249</v>
       </c>
       <c r="T45" s="22">
-        <v>4048</v>
+        <v>4839</v>
       </c>
       <c r="U45" s="19" t="s">
         <v>122</v>
@@ -6380,7 +6380,7 @@
         <v>254</v>
       </c>
       <c r="T46" s="22">
-        <v>4702</v>
+        <v>4664</v>
       </c>
       <c r="U46" s="19" t="s">
         <v>122</v>
@@ -6451,7 +6451,7 @@
         <v>259</v>
       </c>
       <c r="T47" s="22">
-        <v>3953</v>
+        <v>3996</v>
       </c>
       <c r="U47" s="19" t="s">
         <v>122</v>
@@ -6522,7 +6522,7 @@
         <v>266</v>
       </c>
       <c r="T48" s="22">
-        <v>3912</v>
+        <v>6289</v>
       </c>
       <c r="U48" s="19" t="s">
         <v>122</v>
@@ -6593,7 +6593,7 @@
         <v>271</v>
       </c>
       <c r="T49" s="22">
-        <v>5305</v>
+        <v>5162</v>
       </c>
       <c r="U49" s="19" t="s">
         <v>122</v>
@@ -6664,7 +6664,7 @@
         <v>13</v>
       </c>
       <c r="T50" s="22">
-        <v>5918</v>
+        <v>5876</v>
       </c>
       <c r="U50" s="25" t="s">
         <v>135</v>
@@ -6735,7 +6735,7 @@
         <v>13</v>
       </c>
       <c r="T51" s="22">
-        <v>5887</v>
+        <v>5035</v>
       </c>
       <c r="U51" s="25" t="s">
         <v>135</v>

</xml_diff>

<commit_message>
Sprint 2 CI-011 link data export complete
</commit_message>
<xml_diff>
--- a/output/ClubHubInsight.xlsx
+++ b/output/ClubHubInsight.xlsx
@@ -80,13 +80,13 @@
     <t>Crawl Date</t>
   </si>
   <si>
-    <t>02/09/2026, 00:36:22</t>
+    <t>02/09/2026, 09:11:53</t>
   </si>
   <si>
     <t>Crawl Duration</t>
   </si>
   <si>
-    <t>4m 39s</t>
+    <t>4m 28s</t>
   </si>
   <si>
     <t>Version</t>
@@ -137,7 +137,7 @@
     <t>Average Page Load (ms)</t>
   </si>
   <si>
-    <t>5422 ms</t>
+    <t>5192 ms</t>
   </si>
   <si>
     <t>Site Structure</t>
@@ -3258,7 +3258,7 @@
         <v>121</v>
       </c>
       <c r="T2" s="22">
-        <v>4059</v>
+        <v>4452</v>
       </c>
       <c r="U2" s="19" t="s">
         <v>122</v>
@@ -3329,7 +3329,7 @@
         <v>130</v>
       </c>
       <c r="T3" s="22">
-        <v>4003</v>
+        <v>3759</v>
       </c>
       <c r="U3" s="19" t="s">
         <v>122</v>
@@ -3400,7 +3400,7 @@
         <v>13</v>
       </c>
       <c r="T4" s="22">
-        <v>5870</v>
+        <v>5321</v>
       </c>
       <c r="U4" s="25" t="s">
         <v>135</v>
@@ -3471,7 +3471,7 @@
         <v>13</v>
       </c>
       <c r="T5" s="22">
-        <v>5362</v>
+        <v>5295</v>
       </c>
       <c r="U5" s="25" t="s">
         <v>135</v>
@@ -3542,7 +3542,7 @@
         <v>13</v>
       </c>
       <c r="T6" s="22">
-        <v>5682</v>
+        <v>4996</v>
       </c>
       <c r="U6" s="25" t="s">
         <v>135</v>
@@ -3613,7 +3613,7 @@
         <v>13</v>
       </c>
       <c r="T7" s="22">
-        <v>4664</v>
+        <v>5222</v>
       </c>
       <c r="U7" s="25" t="s">
         <v>135</v>
@@ -3684,7 +3684,7 @@
         <v>13</v>
       </c>
       <c r="T8" s="22">
-        <v>4303</v>
+        <v>4337</v>
       </c>
       <c r="U8" s="25" t="s">
         <v>135</v>
@@ -3755,7 +3755,7 @@
         <v>13</v>
       </c>
       <c r="T9" s="22">
-        <v>4702</v>
+        <v>4972</v>
       </c>
       <c r="U9" s="25" t="s">
         <v>135</v>
@@ -3826,7 +3826,7 @@
         <v>13</v>
       </c>
       <c r="T10" s="22">
-        <v>5212</v>
+        <v>4178</v>
       </c>
       <c r="U10" s="25" t="s">
         <v>135</v>
@@ -3897,7 +3897,7 @@
         <v>13</v>
       </c>
       <c r="T11" s="22">
-        <v>5280</v>
+        <v>4997</v>
       </c>
       <c r="U11" s="25" t="s">
         <v>135</v>
@@ -3968,7 +3968,7 @@
         <v>160</v>
       </c>
       <c r="T12" s="22">
-        <v>4719</v>
+        <v>3885</v>
       </c>
       <c r="U12" s="19" t="s">
         <v>122</v>
@@ -4039,7 +4039,7 @@
         <v>13</v>
       </c>
       <c r="T13" s="22">
-        <v>4092</v>
+        <v>3971</v>
       </c>
       <c r="U13" s="25" t="s">
         <v>135</v>
@@ -4110,7 +4110,7 @@
         <v>13</v>
       </c>
       <c r="T14" s="22">
-        <v>5277</v>
+        <v>4965</v>
       </c>
       <c r="U14" s="25" t="s">
         <v>135</v>
@@ -4181,7 +4181,7 @@
         <v>168</v>
       </c>
       <c r="T15" s="22">
-        <v>4939</v>
+        <v>3992</v>
       </c>
       <c r="U15" s="19" t="s">
         <v>122</v>
@@ -4252,7 +4252,7 @@
         <v>13</v>
       </c>
       <c r="T16" s="22">
-        <v>5978</v>
+        <v>5182</v>
       </c>
       <c r="U16" s="25" t="s">
         <v>135</v>
@@ -4323,7 +4323,7 @@
         <v>13</v>
       </c>
       <c r="T17" s="22">
-        <v>4866</v>
+        <v>4924</v>
       </c>
       <c r="U17" s="25" t="s">
         <v>135</v>
@@ -4394,7 +4394,7 @@
         <v>13</v>
       </c>
       <c r="T18" s="22">
-        <v>5417</v>
+        <v>4973</v>
       </c>
       <c r="U18" s="25" t="s">
         <v>135</v>
@@ -4465,7 +4465,7 @@
         <v>13</v>
       </c>
       <c r="T19" s="22">
-        <v>5441</v>
+        <v>5016</v>
       </c>
       <c r="U19" s="25" t="s">
         <v>135</v>
@@ -4536,7 +4536,7 @@
         <v>13</v>
       </c>
       <c r="T20" s="22">
-        <v>4953</v>
+        <v>6522</v>
       </c>
       <c r="U20" s="25" t="s">
         <v>135</v>
@@ -4607,7 +4607,7 @@
         <v>13</v>
       </c>
       <c r="T21" s="22">
-        <v>3836</v>
+        <v>3672</v>
       </c>
       <c r="U21" s="25" t="s">
         <v>135</v>
@@ -4678,7 +4678,7 @@
         <v>13</v>
       </c>
       <c r="T22" s="22">
-        <v>5569</v>
+        <v>4819</v>
       </c>
       <c r="U22" s="25" t="s">
         <v>135</v>
@@ -4749,7 +4749,7 @@
         <v>13</v>
       </c>
       <c r="T23" s="22">
-        <v>4554</v>
+        <v>5044</v>
       </c>
       <c r="U23" s="25" t="s">
         <v>135</v>
@@ -4820,7 +4820,7 @@
         <v>13</v>
       </c>
       <c r="T24" s="22">
-        <v>4854</v>
+        <v>4204</v>
       </c>
       <c r="U24" s="25" t="s">
         <v>135</v>
@@ -4891,7 +4891,7 @@
         <v>13</v>
       </c>
       <c r="T25" s="22">
-        <v>5357</v>
+        <v>4622</v>
       </c>
       <c r="U25" s="25" t="s">
         <v>135</v>
@@ -4962,7 +4962,7 @@
         <v>13</v>
       </c>
       <c r="T26" s="22">
-        <v>5179</v>
+        <v>5303</v>
       </c>
       <c r="U26" s="25" t="s">
         <v>135</v>
@@ -5033,7 +5033,7 @@
         <v>13</v>
       </c>
       <c r="T27" s="22">
-        <v>4988</v>
+        <v>4938</v>
       </c>
       <c r="U27" s="25" t="s">
         <v>135</v>
@@ -5104,7 +5104,7 @@
         <v>13</v>
       </c>
       <c r="T28" s="22">
-        <v>4653</v>
+        <v>3738</v>
       </c>
       <c r="U28" s="25" t="s">
         <v>135</v>
@@ -5175,7 +5175,7 @@
         <v>200</v>
       </c>
       <c r="T29" s="22">
-        <v>4242</v>
+        <v>3916</v>
       </c>
       <c r="U29" s="19" t="s">
         <v>122</v>
@@ -5246,7 +5246,7 @@
         <v>13</v>
       </c>
       <c r="T30" s="22">
-        <v>5270</v>
+        <v>4124</v>
       </c>
       <c r="U30" s="25" t="s">
         <v>135</v>
@@ -5317,7 +5317,7 @@
         <v>13</v>
       </c>
       <c r="T31" s="22">
-        <v>4931</v>
+        <v>5227</v>
       </c>
       <c r="U31" s="25" t="s">
         <v>135</v>
@@ -5388,7 +5388,7 @@
         <v>13</v>
       </c>
       <c r="T32" s="22">
-        <v>4343</v>
+        <v>4266</v>
       </c>
       <c r="U32" s="25" t="s">
         <v>135</v>
@@ -5459,7 +5459,7 @@
         <v>13</v>
       </c>
       <c r="T33" s="22">
-        <v>5505</v>
+        <v>7441</v>
       </c>
       <c r="U33" s="25" t="s">
         <v>135</v>
@@ -5530,7 +5530,7 @@
         <v>13</v>
       </c>
       <c r="T34" s="22">
-        <v>5367</v>
+        <v>5502</v>
       </c>
       <c r="U34" s="25" t="s">
         <v>135</v>
@@ -5601,7 +5601,7 @@
         <v>13</v>
       </c>
       <c r="T35" s="22">
-        <v>5118</v>
+        <v>5268</v>
       </c>
       <c r="U35" s="25" t="s">
         <v>135</v>
@@ -5672,7 +5672,7 @@
         <v>13</v>
       </c>
       <c r="T36" s="22">
-        <v>4056</v>
+        <v>4000</v>
       </c>
       <c r="U36" s="25" t="s">
         <v>135</v>
@@ -5743,7 +5743,7 @@
         <v>13</v>
       </c>
       <c r="T37" s="22">
-        <v>5277</v>
+        <v>4484</v>
       </c>
       <c r="U37" s="25" t="s">
         <v>135</v>
@@ -5812,7 +5812,7 @@
         <v>13</v>
       </c>
       <c r="T38" s="22">
-        <v>30120</v>
+        <v>30113</v>
       </c>
       <c r="U38" s="25" t="s">
         <v>135</v>
@@ -5883,7 +5883,7 @@
         <v>13</v>
       </c>
       <c r="T39" s="22">
-        <v>5059</v>
+        <v>5302</v>
       </c>
       <c r="U39" s="25" t="s">
         <v>135</v>
@@ -5954,7 +5954,7 @@
         <v>225</v>
       </c>
       <c r="T40" s="22">
-        <v>4059</v>
+        <v>4882</v>
       </c>
       <c r="U40" s="19" t="s">
         <v>122</v>
@@ -6025,7 +6025,7 @@
         <v>229</v>
       </c>
       <c r="T41" s="22">
-        <v>4685</v>
+        <v>3991</v>
       </c>
       <c r="U41" s="19" t="s">
         <v>122</v>
@@ -6096,7 +6096,7 @@
         <v>234</v>
       </c>
       <c r="T42" s="22">
-        <v>4863</v>
+        <v>4455</v>
       </c>
       <c r="U42" s="19" t="s">
         <v>122</v>
@@ -6167,7 +6167,7 @@
         <v>238</v>
       </c>
       <c r="T43" s="22">
-        <v>4315</v>
+        <v>4739</v>
       </c>
       <c r="U43" s="19" t="s">
         <v>122</v>
@@ -6238,7 +6238,7 @@
         <v>242</v>
       </c>
       <c r="T44" s="22">
-        <v>4210</v>
+        <v>3949</v>
       </c>
       <c r="U44" s="19" t="s">
         <v>122</v>
@@ -6309,7 +6309,7 @@
         <v>249</v>
       </c>
       <c r="T45" s="22">
-        <v>4839</v>
+        <v>3853</v>
       </c>
       <c r="U45" s="19" t="s">
         <v>122</v>
@@ -6380,7 +6380,7 @@
         <v>254</v>
       </c>
       <c r="T46" s="22">
-        <v>4664</v>
+        <v>4084</v>
       </c>
       <c r="U46" s="19" t="s">
         <v>122</v>
@@ -6451,7 +6451,7 @@
         <v>259</v>
       </c>
       <c r="T47" s="22">
-        <v>3996</v>
+        <v>3787</v>
       </c>
       <c r="U47" s="19" t="s">
         <v>122</v>
@@ -6522,7 +6522,7 @@
         <v>266</v>
       </c>
       <c r="T48" s="22">
-        <v>6289</v>
+        <v>3835</v>
       </c>
       <c r="U48" s="19" t="s">
         <v>122</v>
@@ -6593,7 +6593,7 @@
         <v>271</v>
       </c>
       <c r="T49" s="22">
-        <v>5162</v>
+        <v>4360</v>
       </c>
       <c r="U49" s="19" t="s">
         <v>122</v>
@@ -6664,7 +6664,7 @@
         <v>13</v>
       </c>
       <c r="T50" s="22">
-        <v>5876</v>
+        <v>5694</v>
       </c>
       <c r="U50" s="25" t="s">
         <v>135</v>
@@ -6735,7 +6735,7 @@
         <v>13</v>
       </c>
       <c r="T51" s="22">
-        <v>5035</v>
+        <v>5023</v>
       </c>
       <c r="U51" s="25" t="s">
         <v>135</v>

</xml_diff>

<commit_message>
Sprint 2 CI-011 most referenced complete
</commit_message>
<xml_diff>
--- a/output/ClubHubInsight.xlsx
+++ b/output/ClubHubInsight.xlsx
@@ -80,13 +80,13 @@
     <t>Crawl Date</t>
   </si>
   <si>
-    <t>02/09/2026, 09:11:53</t>
+    <t>02/09/2026, 10:00:58</t>
   </si>
   <si>
     <t>Crawl Duration</t>
   </si>
   <si>
-    <t>4m 28s</t>
+    <t>4m 33s</t>
   </si>
   <si>
     <t>Version</t>
@@ -137,7 +137,7 @@
     <t>Average Page Load (ms)</t>
   </si>
   <si>
-    <t>5192 ms</t>
+    <t>5289 ms</t>
   </si>
   <si>
     <t>Site Structure</t>
@@ -3231,7 +3231,7 @@
         <v>13</v>
       </c>
       <c r="K2" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L2" s="20">
         <v>59</v>
@@ -3258,7 +3258,7 @@
         <v>121</v>
       </c>
       <c r="T2" s="22">
-        <v>4452</v>
+        <v>4744</v>
       </c>
       <c r="U2" s="19" t="s">
         <v>122</v>
@@ -3302,7 +3302,7 @@
         <v>13</v>
       </c>
       <c r="K3" s="20">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="L3" s="20">
         <v>48</v>
@@ -3329,7 +3329,7 @@
         <v>130</v>
       </c>
       <c r="T3" s="22">
-        <v>3759</v>
+        <v>3734</v>
       </c>
       <c r="U3" s="19" t="s">
         <v>122</v>
@@ -3373,7 +3373,7 @@
         <v>13</v>
       </c>
       <c r="K4" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L4" s="20">
         <v>75</v>
@@ -3400,7 +3400,7 @@
         <v>13</v>
       </c>
       <c r="T4" s="22">
-        <v>5321</v>
+        <v>4348</v>
       </c>
       <c r="U4" s="25" t="s">
         <v>135</v>
@@ -3444,7 +3444,7 @@
         <v>13</v>
       </c>
       <c r="K5" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L5" s="20">
         <v>66</v>
@@ -3471,7 +3471,7 @@
         <v>13</v>
       </c>
       <c r="T5" s="22">
-        <v>5295</v>
+        <v>5320</v>
       </c>
       <c r="U5" s="25" t="s">
         <v>135</v>
@@ -3515,7 +3515,7 @@
         <v>13</v>
       </c>
       <c r="K6" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L6" s="20">
         <v>61</v>
@@ -3542,7 +3542,7 @@
         <v>13</v>
       </c>
       <c r="T6" s="22">
-        <v>4996</v>
+        <v>4903</v>
       </c>
       <c r="U6" s="25" t="s">
         <v>135</v>
@@ -3586,7 +3586,7 @@
         <v>13</v>
       </c>
       <c r="K7" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L7" s="20">
         <v>58</v>
@@ -3613,7 +3613,7 @@
         <v>13</v>
       </c>
       <c r="T7" s="22">
-        <v>5222</v>
+        <v>4431</v>
       </c>
       <c r="U7" s="25" t="s">
         <v>135</v>
@@ -3657,7 +3657,7 @@
         <v>13</v>
       </c>
       <c r="K8" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L8" s="20">
         <v>62</v>
@@ -3684,7 +3684,7 @@
         <v>13</v>
       </c>
       <c r="T8" s="22">
-        <v>4337</v>
+        <v>4874</v>
       </c>
       <c r="U8" s="25" t="s">
         <v>135</v>
@@ -3728,7 +3728,7 @@
         <v>13</v>
       </c>
       <c r="K9" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L9" s="20">
         <v>56</v>
@@ -3755,7 +3755,7 @@
         <v>13</v>
       </c>
       <c r="T9" s="22">
-        <v>4972</v>
+        <v>4137</v>
       </c>
       <c r="U9" s="25" t="s">
         <v>135</v>
@@ -3799,7 +3799,7 @@
         <v>13</v>
       </c>
       <c r="K10" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L10" s="20">
         <v>55</v>
@@ -3826,7 +3826,7 @@
         <v>13</v>
       </c>
       <c r="T10" s="22">
-        <v>4178</v>
+        <v>4192</v>
       </c>
       <c r="U10" s="25" t="s">
         <v>135</v>
@@ -3870,7 +3870,7 @@
         <v>13</v>
       </c>
       <c r="K11" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L11" s="20">
         <v>56</v>
@@ -3897,7 +3897,7 @@
         <v>13</v>
       </c>
       <c r="T11" s="22">
-        <v>4997</v>
+        <v>4285</v>
       </c>
       <c r="U11" s="25" t="s">
         <v>135</v>
@@ -3941,7 +3941,7 @@
         <v>13</v>
       </c>
       <c r="K12" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L12" s="20">
         <v>70</v>
@@ -3968,7 +3968,7 @@
         <v>160</v>
       </c>
       <c r="T12" s="22">
-        <v>3885</v>
+        <v>3800</v>
       </c>
       <c r="U12" s="19" t="s">
         <v>122</v>
@@ -4012,7 +4012,7 @@
         <v>13</v>
       </c>
       <c r="K13" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L13" s="20">
         <v>60</v>
@@ -4039,7 +4039,7 @@
         <v>13</v>
       </c>
       <c r="T13" s="22">
-        <v>3971</v>
+        <v>3898</v>
       </c>
       <c r="U13" s="25" t="s">
         <v>135</v>
@@ -4083,7 +4083,7 @@
         <v>13</v>
       </c>
       <c r="K14" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L14" s="20">
         <v>56</v>
@@ -4110,7 +4110,7 @@
         <v>13</v>
       </c>
       <c r="T14" s="22">
-        <v>4965</v>
+        <v>5053</v>
       </c>
       <c r="U14" s="25" t="s">
         <v>135</v>
@@ -4154,7 +4154,7 @@
         <v>13</v>
       </c>
       <c r="K15" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L15" s="20">
         <v>85</v>
@@ -4181,7 +4181,7 @@
         <v>168</v>
       </c>
       <c r="T15" s="22">
-        <v>3992</v>
+        <v>4077</v>
       </c>
       <c r="U15" s="19" t="s">
         <v>122</v>
@@ -4225,7 +4225,7 @@
         <v>13</v>
       </c>
       <c r="K16" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L16" s="20">
         <v>59</v>
@@ -4252,7 +4252,7 @@
         <v>13</v>
       </c>
       <c r="T16" s="22">
-        <v>5182</v>
+        <v>5152</v>
       </c>
       <c r="U16" s="25" t="s">
         <v>135</v>
@@ -4296,7 +4296,7 @@
         <v>13</v>
       </c>
       <c r="K17" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L17" s="20">
         <v>57</v>
@@ -4323,7 +4323,7 @@
         <v>13</v>
       </c>
       <c r="T17" s="22">
-        <v>4924</v>
+        <v>4767</v>
       </c>
       <c r="U17" s="25" t="s">
         <v>135</v>
@@ -4367,7 +4367,7 @@
         <v>13</v>
       </c>
       <c r="K18" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L18" s="20">
         <v>82</v>
@@ -4394,7 +4394,7 @@
         <v>13</v>
       </c>
       <c r="T18" s="22">
-        <v>4973</v>
+        <v>5044</v>
       </c>
       <c r="U18" s="25" t="s">
         <v>135</v>
@@ -4438,7 +4438,7 @@
         <v>13</v>
       </c>
       <c r="K19" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L19" s="20">
         <v>63</v>
@@ -4465,7 +4465,7 @@
         <v>13</v>
       </c>
       <c r="T19" s="22">
-        <v>5016</v>
+        <v>6319</v>
       </c>
       <c r="U19" s="25" t="s">
         <v>135</v>
@@ -4509,7 +4509,7 @@
         <v>13</v>
       </c>
       <c r="K20" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L20" s="20">
         <v>53</v>
@@ -4536,7 +4536,7 @@
         <v>13</v>
       </c>
       <c r="T20" s="22">
-        <v>6522</v>
+        <v>5008</v>
       </c>
       <c r="U20" s="25" t="s">
         <v>135</v>
@@ -4580,7 +4580,7 @@
         <v>13</v>
       </c>
       <c r="K21" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L21" s="20">
         <v>48</v>
@@ -4607,7 +4607,7 @@
         <v>13</v>
       </c>
       <c r="T21" s="22">
-        <v>3672</v>
+        <v>5295</v>
       </c>
       <c r="U21" s="25" t="s">
         <v>135</v>
@@ -4651,7 +4651,7 @@
         <v>13</v>
       </c>
       <c r="K22" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L22" s="20">
         <v>51</v>
@@ -4678,7 +4678,7 @@
         <v>13</v>
       </c>
       <c r="T22" s="22">
-        <v>4819</v>
+        <v>4227</v>
       </c>
       <c r="U22" s="25" t="s">
         <v>135</v>
@@ -4722,7 +4722,7 @@
         <v>13</v>
       </c>
       <c r="K23" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L23" s="20">
         <v>53</v>
@@ -4749,7 +4749,7 @@
         <v>13</v>
       </c>
       <c r="T23" s="22">
-        <v>5044</v>
+        <v>4315</v>
       </c>
       <c r="U23" s="25" t="s">
         <v>135</v>
@@ -4793,7 +4793,7 @@
         <v>13</v>
       </c>
       <c r="K24" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L24" s="20">
         <v>75</v>
@@ -4820,7 +4820,7 @@
         <v>13</v>
       </c>
       <c r="T24" s="22">
-        <v>4204</v>
+        <v>4426</v>
       </c>
       <c r="U24" s="25" t="s">
         <v>135</v>
@@ -4864,7 +4864,7 @@
         <v>13</v>
       </c>
       <c r="K25" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L25" s="20">
         <v>60</v>
@@ -4891,7 +4891,7 @@
         <v>13</v>
       </c>
       <c r="T25" s="22">
-        <v>4622</v>
+        <v>4517</v>
       </c>
       <c r="U25" s="25" t="s">
         <v>135</v>
@@ -4935,7 +4935,7 @@
         <v>13</v>
       </c>
       <c r="K26" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L26" s="20">
         <v>60</v>
@@ -4962,7 +4962,7 @@
         <v>13</v>
       </c>
       <c r="T26" s="22">
-        <v>5303</v>
+        <v>4651</v>
       </c>
       <c r="U26" s="25" t="s">
         <v>135</v>
@@ -5006,7 +5006,7 @@
         <v>13</v>
       </c>
       <c r="K27" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L27" s="20">
         <v>54</v>
@@ -5033,7 +5033,7 @@
         <v>13</v>
       </c>
       <c r="T27" s="22">
-        <v>4938</v>
+        <v>4433</v>
       </c>
       <c r="U27" s="25" t="s">
         <v>135</v>
@@ -5077,7 +5077,7 @@
         <v>13</v>
       </c>
       <c r="K28" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L28" s="20">
         <v>52</v>
@@ -5104,7 +5104,7 @@
         <v>13</v>
       </c>
       <c r="T28" s="22">
-        <v>3738</v>
+        <v>6486</v>
       </c>
       <c r="U28" s="25" t="s">
         <v>135</v>
@@ -5148,7 +5148,7 @@
         <v>13</v>
       </c>
       <c r="K29" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L29" s="20">
         <v>59</v>
@@ -5175,7 +5175,7 @@
         <v>200</v>
       </c>
       <c r="T29" s="22">
-        <v>3916</v>
+        <v>4514</v>
       </c>
       <c r="U29" s="19" t="s">
         <v>122</v>
@@ -5219,7 +5219,7 @@
         <v>13</v>
       </c>
       <c r="K30" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L30" s="20">
         <v>118</v>
@@ -5246,7 +5246,7 @@
         <v>13</v>
       </c>
       <c r="T30" s="22">
-        <v>4124</v>
+        <v>4793</v>
       </c>
       <c r="U30" s="25" t="s">
         <v>135</v>
@@ -5290,7 +5290,7 @@
         <v>13</v>
       </c>
       <c r="K31" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L31" s="20">
         <v>76</v>
@@ -5317,7 +5317,7 @@
         <v>13</v>
       </c>
       <c r="T31" s="22">
-        <v>5227</v>
+        <v>4360</v>
       </c>
       <c r="U31" s="25" t="s">
         <v>135</v>
@@ -5361,7 +5361,7 @@
         <v>13</v>
       </c>
       <c r="K32" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L32" s="20">
         <v>72</v>
@@ -5388,7 +5388,7 @@
         <v>13</v>
       </c>
       <c r="T32" s="22">
-        <v>4266</v>
+        <v>4287</v>
       </c>
       <c r="U32" s="25" t="s">
         <v>135</v>
@@ -5432,7 +5432,7 @@
         <v>13</v>
       </c>
       <c r="K33" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L33" s="20">
         <v>66</v>
@@ -5459,7 +5459,7 @@
         <v>13</v>
       </c>
       <c r="T33" s="22">
-        <v>7441</v>
+        <v>5844</v>
       </c>
       <c r="U33" s="25" t="s">
         <v>135</v>
@@ -5503,7 +5503,7 @@
         <v>13</v>
       </c>
       <c r="K34" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L34" s="20">
         <v>68</v>
@@ -5530,7 +5530,7 @@
         <v>13</v>
       </c>
       <c r="T34" s="22">
-        <v>5502</v>
+        <v>5046</v>
       </c>
       <c r="U34" s="25" t="s">
         <v>135</v>
@@ -5574,7 +5574,7 @@
         <v>13</v>
       </c>
       <c r="K35" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L35" s="20">
         <v>62</v>
@@ -5601,7 +5601,7 @@
         <v>13</v>
       </c>
       <c r="T35" s="22">
-        <v>5268</v>
+        <v>4914</v>
       </c>
       <c r="U35" s="25" t="s">
         <v>135</v>
@@ -5645,7 +5645,7 @@
         <v>13</v>
       </c>
       <c r="K36" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L36" s="20">
         <v>56</v>
@@ -5672,7 +5672,7 @@
         <v>13</v>
       </c>
       <c r="T36" s="22">
-        <v>4000</v>
+        <v>4270</v>
       </c>
       <c r="U36" s="25" t="s">
         <v>135</v>
@@ -5716,7 +5716,7 @@
         <v>13</v>
       </c>
       <c r="K37" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L37" s="20">
         <v>61</v>
@@ -5743,7 +5743,7 @@
         <v>13</v>
       </c>
       <c r="T37" s="22">
-        <v>4484</v>
+        <v>4394</v>
       </c>
       <c r="U37" s="25" t="s">
         <v>135</v>
@@ -5812,7 +5812,7 @@
         <v>13</v>
       </c>
       <c r="T38" s="22">
-        <v>30113</v>
+        <v>30112</v>
       </c>
       <c r="U38" s="25" t="s">
         <v>135</v>
@@ -5856,7 +5856,7 @@
         <v>13</v>
       </c>
       <c r="K39" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L39" s="20">
         <v>61</v>
@@ -5883,7 +5883,7 @@
         <v>13</v>
       </c>
       <c r="T39" s="22">
-        <v>5302</v>
+        <v>5172</v>
       </c>
       <c r="U39" s="25" t="s">
         <v>135</v>
@@ -5927,7 +5927,7 @@
         <v>13</v>
       </c>
       <c r="K40" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L40" s="20">
         <v>47</v>
@@ -5954,7 +5954,7 @@
         <v>225</v>
       </c>
       <c r="T40" s="22">
-        <v>4882</v>
+        <v>4501</v>
       </c>
       <c r="U40" s="19" t="s">
         <v>122</v>
@@ -5998,7 +5998,7 @@
         <v>13</v>
       </c>
       <c r="K41" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L41" s="20">
         <v>47</v>
@@ -6025,7 +6025,7 @@
         <v>229</v>
       </c>
       <c r="T41" s="22">
-        <v>3991</v>
+        <v>9521</v>
       </c>
       <c r="U41" s="19" t="s">
         <v>122</v>
@@ -6069,7 +6069,7 @@
         <v>13</v>
       </c>
       <c r="K42" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L42" s="20">
         <v>47</v>
@@ -6096,7 +6096,7 @@
         <v>234</v>
       </c>
       <c r="T42" s="22">
-        <v>4455</v>
+        <v>5438</v>
       </c>
       <c r="U42" s="19" t="s">
         <v>122</v>
@@ -6140,7 +6140,7 @@
         <v>13</v>
       </c>
       <c r="K43" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L43" s="20">
         <v>47</v>
@@ -6167,7 +6167,7 @@
         <v>238</v>
       </c>
       <c r="T43" s="22">
-        <v>4739</v>
+        <v>4255</v>
       </c>
       <c r="U43" s="19" t="s">
         <v>122</v>
@@ -6211,7 +6211,7 @@
         <v>13</v>
       </c>
       <c r="K44" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L44" s="20">
         <v>47</v>
@@ -6238,7 +6238,7 @@
         <v>242</v>
       </c>
       <c r="T44" s="22">
-        <v>3949</v>
+        <v>4275</v>
       </c>
       <c r="U44" s="19" t="s">
         <v>122</v>
@@ -6282,7 +6282,7 @@
         <v>13</v>
       </c>
       <c r="K45" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L45" s="20">
         <v>57</v>
@@ -6309,7 +6309,7 @@
         <v>249</v>
       </c>
       <c r="T45" s="22">
-        <v>3853</v>
+        <v>4196</v>
       </c>
       <c r="U45" s="19" t="s">
         <v>122</v>
@@ -6353,7 +6353,7 @@
         <v>13</v>
       </c>
       <c r="K46" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L46" s="20">
         <v>52</v>
@@ -6380,7 +6380,7 @@
         <v>254</v>
       </c>
       <c r="T46" s="22">
-        <v>4084</v>
+        <v>3850</v>
       </c>
       <c r="U46" s="19" t="s">
         <v>122</v>
@@ -6424,7 +6424,7 @@
         <v>13</v>
       </c>
       <c r="K47" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L47" s="20">
         <v>47</v>
@@ -6451,7 +6451,7 @@
         <v>259</v>
       </c>
       <c r="T47" s="22">
-        <v>3787</v>
+        <v>3915</v>
       </c>
       <c r="U47" s="19" t="s">
         <v>122</v>
@@ -6495,7 +6495,7 @@
         <v>13</v>
       </c>
       <c r="K48" s="20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L48" s="20">
         <v>47</v>
@@ -6522,7 +6522,7 @@
         <v>266</v>
       </c>
       <c r="T48" s="22">
-        <v>3835</v>
+        <v>4945</v>
       </c>
       <c r="U48" s="19" t="s">
         <v>122</v>
@@ -6566,7 +6566,7 @@
         <v>13</v>
       </c>
       <c r="K49" s="20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L49" s="20">
         <v>68</v>
@@ -6593,7 +6593,7 @@
         <v>271</v>
       </c>
       <c r="T49" s="22">
-        <v>4360</v>
+        <v>4877</v>
       </c>
       <c r="U49" s="19" t="s">
         <v>122</v>
@@ -6637,7 +6637,7 @@
         <v>13</v>
       </c>
       <c r="K50" s="20">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="L50" s="20">
         <v>68</v>
@@ -6664,7 +6664,7 @@
         <v>13</v>
       </c>
       <c r="T50" s="22">
-        <v>5694</v>
+        <v>5344</v>
       </c>
       <c r="U50" s="25" t="s">
         <v>135</v>
@@ -6708,7 +6708,7 @@
         <v>13</v>
       </c>
       <c r="K51" s="20">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L51" s="20">
         <v>70</v>
@@ -6735,7 +6735,7 @@
         <v>13</v>
       </c>
       <c r="T51" s="22">
-        <v>5023</v>
+        <v>5186</v>
       </c>
       <c r="U51" s="25" t="s">
         <v>135</v>
@@ -7875,7 +7875,7 @@
         <v>113</v>
       </c>
       <c r="C2">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D2">
         <v>59</v>
@@ -7892,7 +7892,7 @@
         <v>125</v>
       </c>
       <c r="C3">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D3">
         <v>48</v>
@@ -7909,7 +7909,7 @@
         <v>132</v>
       </c>
       <c r="C4">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D4">
         <v>75</v>
@@ -7926,7 +7926,7 @@
         <v>138</v>
       </c>
       <c r="C5">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D5">
         <v>66</v>
@@ -7943,7 +7943,7 @@
         <v>142</v>
       </c>
       <c r="C6">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D6">
         <v>61</v>
@@ -7960,7 +7960,7 @@
         <v>144</v>
       </c>
       <c r="C7">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D7">
         <v>58</v>
@@ -7977,7 +7977,7 @@
         <v>147</v>
       </c>
       <c r="C8">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D8">
         <v>62</v>
@@ -7994,7 +7994,7 @@
         <v>150</v>
       </c>
       <c r="C9">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D9">
         <v>56</v>
@@ -8011,7 +8011,7 @@
         <v>153</v>
       </c>
       <c r="C10">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D10">
         <v>55</v>
@@ -8028,7 +8028,7 @@
         <v>155</v>
       </c>
       <c r="C11">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D11">
         <v>56</v>
@@ -8045,7 +8045,7 @@
         <v>157</v>
       </c>
       <c r="C12">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D12">
         <v>70</v>
@@ -8062,7 +8062,7 @@
         <v>162</v>
       </c>
       <c r="C13">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D13">
         <v>60</v>
@@ -8079,7 +8079,7 @@
         <v>164</v>
       </c>
       <c r="C14">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D14">
         <v>56</v>
@@ -8096,7 +8096,7 @@
         <v>166</v>
       </c>
       <c r="C15">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D15">
         <v>85</v>
@@ -8113,7 +8113,7 @@
         <v>170</v>
       </c>
       <c r="C16">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D16">
         <v>59</v>
@@ -8130,7 +8130,7 @@
         <v>172</v>
       </c>
       <c r="C17">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D17">
         <v>57</v>
@@ -8147,7 +8147,7 @@
         <v>139</v>
       </c>
       <c r="C18">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D18">
         <v>82</v>
@@ -8164,7 +8164,7 @@
         <v>176</v>
       </c>
       <c r="C19">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D19">
         <v>63</v>
@@ -8181,7 +8181,7 @@
         <v>178</v>
       </c>
       <c r="C20">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D20">
         <v>53</v>
@@ -8198,7 +8198,7 @@
         <v>180</v>
       </c>
       <c r="C21">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D21">
         <v>48</v>
@@ -8215,7 +8215,7 @@
         <v>184</v>
       </c>
       <c r="C22">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D22">
         <v>51</v>
@@ -8232,7 +8232,7 @@
         <v>186</v>
       </c>
       <c r="C23">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D23">
         <v>53</v>
@@ -8249,7 +8249,7 @@
         <v>188</v>
       </c>
       <c r="C24">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D24">
         <v>75</v>
@@ -8266,7 +8266,7 @@
         <v>190</v>
       </c>
       <c r="C25">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D25">
         <v>60</v>
@@ -8283,7 +8283,7 @@
         <v>192</v>
       </c>
       <c r="C26">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D26">
         <v>60</v>
@@ -8300,7 +8300,7 @@
         <v>194</v>
       </c>
       <c r="C27">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D27">
         <v>54</v>
@@ -8317,7 +8317,7 @@
         <v>196</v>
       </c>
       <c r="C28">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D28">
         <v>52</v>
@@ -8334,7 +8334,7 @@
         <v>198</v>
       </c>
       <c r="C29">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D29">
         <v>59</v>
@@ -8351,7 +8351,7 @@
         <v>202</v>
       </c>
       <c r="C30">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D30">
         <v>118</v>
@@ -8368,7 +8368,7 @@
         <v>204</v>
       </c>
       <c r="C31">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D31">
         <v>76</v>
@@ -8385,7 +8385,7 @@
         <v>145</v>
       </c>
       <c r="C32">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D32">
         <v>72</v>
@@ -8402,7 +8402,7 @@
         <v>208</v>
       </c>
       <c r="C33">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D33">
         <v>66</v>
@@ -8419,7 +8419,7 @@
         <v>210</v>
       </c>
       <c r="C34">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D34">
         <v>68</v>
@@ -8436,7 +8436,7 @@
         <v>212</v>
       </c>
       <c r="C35">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D35">
         <v>62</v>
@@ -8453,7 +8453,7 @@
         <v>214</v>
       </c>
       <c r="C36">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D36">
         <v>56</v>
@@ -8470,7 +8470,7 @@
         <v>216</v>
       </c>
       <c r="C37">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D37">
         <v>61</v>
@@ -8504,7 +8504,7 @@
         <v>220</v>
       </c>
       <c r="C39">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D39">
         <v>61</v>
@@ -8521,7 +8521,7 @@
         <v>222</v>
       </c>
       <c r="C40">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D40">
         <v>47</v>
@@ -8538,7 +8538,7 @@
         <v>227</v>
       </c>
       <c r="C41">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D41">
         <v>47</v>
@@ -8555,7 +8555,7 @@
         <v>231</v>
       </c>
       <c r="C42">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D42">
         <v>47</v>
@@ -8572,7 +8572,7 @@
         <v>236</v>
       </c>
       <c r="C43">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D43">
         <v>47</v>
@@ -8589,7 +8589,7 @@
         <v>240</v>
       </c>
       <c r="C44">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D44">
         <v>47</v>
@@ -8606,7 +8606,7 @@
         <v>244</v>
       </c>
       <c r="C45">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D45">
         <v>57</v>
@@ -8623,7 +8623,7 @@
         <v>251</v>
       </c>
       <c r="C46">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D46">
         <v>52</v>
@@ -8640,7 +8640,7 @@
         <v>256</v>
       </c>
       <c r="C47">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D47">
         <v>47</v>
@@ -8657,7 +8657,7 @@
         <v>261</v>
       </c>
       <c r="C48">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D48">
         <v>47</v>
@@ -8674,7 +8674,7 @@
         <v>268</v>
       </c>
       <c r="C49">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D49">
         <v>68</v>
@@ -8691,7 +8691,7 @@
         <v>273</v>
       </c>
       <c r="C50">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D50">
         <v>68</v>
@@ -8708,7 +8708,7 @@
         <v>275</v>
       </c>
       <c r="C51">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D51">
         <v>70</v>

</xml_diff>

<commit_message>
Sprint 2 CI-003 explain metrics complete
</commit_message>
<xml_diff>
--- a/output/ClubHubInsight.xlsx
+++ b/output/ClubHubInsight.xlsx
@@ -82,13 +82,13 @@
     <t>Crawl Date</t>
   </si>
   <si>
-    <t>02/09/2026, 11:25:31</t>
+    <t>02/09/2026, 12:15:42</t>
   </si>
   <si>
     <t>Crawl Duration</t>
   </si>
   <si>
-    <t>4m 45s</t>
+    <t>4m 58s</t>
   </si>
   <si>
     <t>Version</t>
@@ -139,7 +139,7 @@
     <t>Average Page Load (ms)</t>
   </si>
   <si>
-    <t>5526 ms</t>
+    <t>5787 ms</t>
   </si>
   <si>
     <t>Site Structure</t>
@@ -3094,7 +3094,7 @@
         <v>323</v>
       </c>
       <c r="C32" s="20">
-        <v>2977</v>
+        <v>2978</v>
       </c>
       <c r="D32" s="37" t="s">
         <v>13</v>
@@ -3833,7 +3833,7 @@
         <v>34</v>
       </c>
       <c r="B27" s="12">
-        <v>2977</v>
+        <v>2978</v>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -4300,7 +4300,7 @@
         <v>121</v>
       </c>
       <c r="T2" s="22">
-        <v>4910</v>
+        <v>5183</v>
       </c>
       <c r="U2" s="19" t="s">
         <v>122</v>
@@ -4371,7 +4371,7 @@
         <v>130</v>
       </c>
       <c r="T3" s="22">
-        <v>4559</v>
+        <v>4980</v>
       </c>
       <c r="U3" s="19" t="s">
         <v>122</v>
@@ -4442,7 +4442,7 @@
         <v>13</v>
       </c>
       <c r="T4" s="22">
-        <v>5475</v>
+        <v>5010</v>
       </c>
       <c r="U4" s="25" t="s">
         <v>135</v>
@@ -4513,7 +4513,7 @@
         <v>13</v>
       </c>
       <c r="T5" s="22">
-        <v>5483</v>
+        <v>5358</v>
       </c>
       <c r="U5" s="25" t="s">
         <v>135</v>
@@ -4584,7 +4584,7 @@
         <v>13</v>
       </c>
       <c r="T6" s="22">
-        <v>5020</v>
+        <v>5058</v>
       </c>
       <c r="U6" s="25" t="s">
         <v>135</v>
@@ -4655,7 +4655,7 @@
         <v>13</v>
       </c>
       <c r="T7" s="22">
-        <v>4534</v>
+        <v>4823</v>
       </c>
       <c r="U7" s="25" t="s">
         <v>135</v>
@@ -4726,7 +4726,7 @@
         <v>13</v>
       </c>
       <c r="T8" s="22">
-        <v>4418</v>
+        <v>6115</v>
       </c>
       <c r="U8" s="25" t="s">
         <v>135</v>
@@ -4797,7 +4797,7 @@
         <v>13</v>
       </c>
       <c r="T9" s="22">
-        <v>5392</v>
+        <v>4484</v>
       </c>
       <c r="U9" s="25" t="s">
         <v>135</v>
@@ -4868,7 +4868,7 @@
         <v>13</v>
       </c>
       <c r="T10" s="22">
-        <v>4989</v>
+        <v>4992</v>
       </c>
       <c r="U10" s="25" t="s">
         <v>135</v>
@@ -4939,7 +4939,7 @@
         <v>13</v>
       </c>
       <c r="T11" s="22">
-        <v>5170</v>
+        <v>4761</v>
       </c>
       <c r="U11" s="25" t="s">
         <v>135</v>
@@ -5010,7 +5010,7 @@
         <v>160</v>
       </c>
       <c r="T12" s="22">
-        <v>4772</v>
+        <v>4269</v>
       </c>
       <c r="U12" s="19" t="s">
         <v>122</v>
@@ -5081,7 +5081,7 @@
         <v>13</v>
       </c>
       <c r="T13" s="22">
-        <v>4146</v>
+        <v>4093</v>
       </c>
       <c r="U13" s="25" t="s">
         <v>135</v>
@@ -5152,7 +5152,7 @@
         <v>13</v>
       </c>
       <c r="T14" s="22">
-        <v>4900</v>
+        <v>5053</v>
       </c>
       <c r="U14" s="25" t="s">
         <v>135</v>
@@ -5223,7 +5223,7 @@
         <v>168</v>
       </c>
       <c r="T15" s="22">
-        <v>5262</v>
+        <v>5367</v>
       </c>
       <c r="U15" s="19" t="s">
         <v>122</v>
@@ -5294,7 +5294,7 @@
         <v>13</v>
       </c>
       <c r="T16" s="22">
-        <v>6788</v>
+        <v>5619</v>
       </c>
       <c r="U16" s="25" t="s">
         <v>135</v>
@@ -5365,7 +5365,7 @@
         <v>13</v>
       </c>
       <c r="T17" s="22">
-        <v>5116</v>
+        <v>4723</v>
       </c>
       <c r="U17" s="25" t="s">
         <v>135</v>
@@ -5436,7 +5436,7 @@
         <v>13</v>
       </c>
       <c r="T18" s="22">
-        <v>5254</v>
+        <v>5272</v>
       </c>
       <c r="U18" s="25" t="s">
         <v>135</v>
@@ -5507,7 +5507,7 @@
         <v>13</v>
       </c>
       <c r="T19" s="22">
-        <v>5422</v>
+        <v>4750</v>
       </c>
       <c r="U19" s="25" t="s">
         <v>135</v>
@@ -5578,7 +5578,7 @@
         <v>13</v>
       </c>
       <c r="T20" s="22">
-        <v>7407</v>
+        <v>5192</v>
       </c>
       <c r="U20" s="25" t="s">
         <v>135</v>
@@ -5649,7 +5649,7 @@
         <v>13</v>
       </c>
       <c r="T21" s="22">
-        <v>3946</v>
+        <v>4059</v>
       </c>
       <c r="U21" s="25" t="s">
         <v>135</v>
@@ -5720,7 +5720,7 @@
         <v>13</v>
       </c>
       <c r="T22" s="22">
-        <v>6183</v>
+        <v>5006</v>
       </c>
       <c r="U22" s="25" t="s">
         <v>135</v>
@@ -5791,7 +5791,7 @@
         <v>13</v>
       </c>
       <c r="T23" s="22">
-        <v>4485</v>
+        <v>5047</v>
       </c>
       <c r="U23" s="25" t="s">
         <v>135</v>
@@ -5862,7 +5862,7 @@
         <v>13</v>
       </c>
       <c r="T24" s="22">
-        <v>4571</v>
+        <v>4737</v>
       </c>
       <c r="U24" s="25" t="s">
         <v>135</v>
@@ -5933,7 +5933,7 @@
         <v>13</v>
       </c>
       <c r="T25" s="22">
-        <v>4754</v>
+        <v>5268</v>
       </c>
       <c r="U25" s="25" t="s">
         <v>135</v>
@@ -6004,7 +6004,7 @@
         <v>13</v>
       </c>
       <c r="T26" s="22">
-        <v>6221</v>
+        <v>4736</v>
       </c>
       <c r="U26" s="25" t="s">
         <v>135</v>
@@ -6075,7 +6075,7 @@
         <v>13</v>
       </c>
       <c r="T27" s="22">
-        <v>4668</v>
+        <v>6288</v>
       </c>
       <c r="U27" s="25" t="s">
         <v>135</v>
@@ -6146,7 +6146,7 @@
         <v>13</v>
       </c>
       <c r="T28" s="22">
-        <v>4658</v>
+        <v>5312</v>
       </c>
       <c r="U28" s="25" t="s">
         <v>135</v>
@@ -6217,7 +6217,7 @@
         <v>200</v>
       </c>
       <c r="T29" s="22">
-        <v>4114</v>
+        <v>4676</v>
       </c>
       <c r="U29" s="19" t="s">
         <v>122</v>
@@ -6288,7 +6288,7 @@
         <v>13</v>
       </c>
       <c r="T30" s="22">
-        <v>4646</v>
+        <v>5026</v>
       </c>
       <c r="U30" s="25" t="s">
         <v>135</v>
@@ -6359,7 +6359,7 @@
         <v>13</v>
       </c>
       <c r="T31" s="22">
-        <v>5480</v>
+        <v>5767</v>
       </c>
       <c r="U31" s="25" t="s">
         <v>135</v>
@@ -6430,7 +6430,7 @@
         <v>13</v>
       </c>
       <c r="T32" s="22">
-        <v>4758</v>
+        <v>4765</v>
       </c>
       <c r="U32" s="25" t="s">
         <v>135</v>
@@ -6501,7 +6501,7 @@
         <v>13</v>
       </c>
       <c r="T33" s="22">
-        <v>5252</v>
+        <v>6760</v>
       </c>
       <c r="U33" s="25" t="s">
         <v>135</v>
@@ -6572,7 +6572,7 @@
         <v>13</v>
       </c>
       <c r="T34" s="22">
-        <v>5485</v>
+        <v>5188</v>
       </c>
       <c r="U34" s="25" t="s">
         <v>135</v>
@@ -6643,7 +6643,7 @@
         <v>13</v>
       </c>
       <c r="T35" s="22">
-        <v>5145</v>
+        <v>5036</v>
       </c>
       <c r="U35" s="25" t="s">
         <v>135</v>
@@ -6714,7 +6714,7 @@
         <v>13</v>
       </c>
       <c r="T36" s="22">
-        <v>4154</v>
+        <v>4245</v>
       </c>
       <c r="U36" s="25" t="s">
         <v>135</v>
@@ -6785,7 +6785,7 @@
         <v>13</v>
       </c>
       <c r="T37" s="22">
-        <v>5074</v>
+        <v>5210</v>
       </c>
       <c r="U37" s="25" t="s">
         <v>135</v>
@@ -6854,7 +6854,7 @@
         <v>13</v>
       </c>
       <c r="T38" s="22">
-        <v>30115</v>
+        <v>30120</v>
       </c>
       <c r="U38" s="25" t="s">
         <v>135</v>
@@ -6925,7 +6925,7 @@
         <v>13</v>
       </c>
       <c r="T39" s="22">
-        <v>5257</v>
+        <v>5780</v>
       </c>
       <c r="U39" s="25" t="s">
         <v>135</v>
@@ -6996,7 +6996,7 @@
         <v>225</v>
       </c>
       <c r="T40" s="22">
-        <v>4272</v>
+        <v>4289</v>
       </c>
       <c r="U40" s="19" t="s">
         <v>122</v>
@@ -7067,7 +7067,7 @@
         <v>229</v>
       </c>
       <c r="T41" s="22">
-        <v>4817</v>
+        <v>4815</v>
       </c>
       <c r="U41" s="19" t="s">
         <v>122</v>
@@ -7138,7 +7138,7 @@
         <v>234</v>
       </c>
       <c r="T42" s="22">
-        <v>5407</v>
+        <v>5047</v>
       </c>
       <c r="U42" s="19" t="s">
         <v>122</v>
@@ -7209,7 +7209,7 @@
         <v>238</v>
       </c>
       <c r="T43" s="22">
-        <v>4570</v>
+        <v>4630</v>
       </c>
       <c r="U43" s="19" t="s">
         <v>122</v>
@@ -7280,7 +7280,7 @@
         <v>242</v>
       </c>
       <c r="T44" s="22">
-        <v>4955</v>
+        <v>4343</v>
       </c>
       <c r="U44" s="19" t="s">
         <v>122</v>
@@ -7351,7 +7351,7 @@
         <v>249</v>
       </c>
       <c r="T45" s="22">
-        <v>4171</v>
+        <v>3993</v>
       </c>
       <c r="U45" s="19" t="s">
         <v>122</v>
@@ -7422,7 +7422,7 @@
         <v>254</v>
       </c>
       <c r="T46" s="22">
-        <v>6170</v>
+        <v>7378</v>
       </c>
       <c r="U46" s="19" t="s">
         <v>122</v>
@@ -7493,7 +7493,7 @@
         <v>259</v>
       </c>
       <c r="T47" s="22">
-        <v>4533</v>
+        <v>4531</v>
       </c>
       <c r="U47" s="19" t="s">
         <v>122</v>
@@ -7564,7 +7564,7 @@
         <v>266</v>
       </c>
       <c r="T48" s="22">
-        <v>3989</v>
+        <v>4468</v>
       </c>
       <c r="U48" s="19" t="s">
         <v>122</v>
@@ -7635,7 +7635,7 @@
         <v>271</v>
       </c>
       <c r="T49" s="22">
-        <v>5028</v>
+        <v>4643</v>
       </c>
       <c r="U49" s="19" t="s">
         <v>122</v>
@@ -7706,7 +7706,7 @@
         <v>13</v>
       </c>
       <c r="T50" s="22">
-        <v>5219</v>
+        <v>5170</v>
       </c>
       <c r="U50" s="25" t="s">
         <v>135</v>
@@ -7753,7 +7753,7 @@
         <v>10</v>
       </c>
       <c r="L51" s="20">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="M51" s="21">
         <v>36</v>
@@ -7777,7 +7777,7 @@
         <v>13</v>
       </c>
       <c r="T51" s="22">
-        <v>5199</v>
+        <v>17909</v>
       </c>
       <c r="U51" s="25" t="s">
         <v>135</v>
@@ -9753,7 +9753,7 @@
         <v>10</v>
       </c>
       <c r="D51">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E51" s="32" t="s">
         <v>282</v>

</xml_diff>

<commit_message>
Sprint 2 CI-004 metric drill-down complete
</commit_message>
<xml_diff>
--- a/output/ClubHubInsight.xlsx
+++ b/output/ClubHubInsight.xlsx
@@ -82,13 +82,13 @@
     <t>Crawl Date</t>
   </si>
   <si>
-    <t>02/09/2026, 12:15:42</t>
+    <t>02/09/2026, 12:58:34</t>
   </si>
   <si>
     <t>Crawl Duration</t>
   </si>
   <si>
-    <t>4m 58s</t>
+    <t>4m 51s</t>
   </si>
   <si>
     <t>Version</t>
@@ -139,7 +139,7 @@
     <t>Average Page Load (ms)</t>
   </si>
   <si>
-    <t>5787 ms</t>
+    <t>5660 ms</t>
   </si>
   <si>
     <t>Site Structure</t>
@@ -3094,7 +3094,7 @@
         <v>323</v>
       </c>
       <c r="C32" s="20">
-        <v>2978</v>
+        <v>2977</v>
       </c>
       <c r="D32" s="37" t="s">
         <v>13</v>
@@ -3833,7 +3833,7 @@
         <v>34</v>
       </c>
       <c r="B27" s="12">
-        <v>2978</v>
+        <v>2977</v>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -4300,7 +4300,7 @@
         <v>121</v>
       </c>
       <c r="T2" s="22">
-        <v>5183</v>
+        <v>4954</v>
       </c>
       <c r="U2" s="19" t="s">
         <v>122</v>
@@ -4371,7 +4371,7 @@
         <v>130</v>
       </c>
       <c r="T3" s="22">
-        <v>4980</v>
+        <v>3815</v>
       </c>
       <c r="U3" s="19" t="s">
         <v>122</v>
@@ -4442,7 +4442,7 @@
         <v>13</v>
       </c>
       <c r="T4" s="22">
-        <v>5010</v>
+        <v>6357</v>
       </c>
       <c r="U4" s="25" t="s">
         <v>135</v>
@@ -4513,7 +4513,7 @@
         <v>13</v>
       </c>
       <c r="T5" s="22">
-        <v>5358</v>
+        <v>5777</v>
       </c>
       <c r="U5" s="25" t="s">
         <v>135</v>
@@ -4584,7 +4584,7 @@
         <v>13</v>
       </c>
       <c r="T6" s="22">
-        <v>5058</v>
+        <v>5061</v>
       </c>
       <c r="U6" s="25" t="s">
         <v>135</v>
@@ -4655,7 +4655,7 @@
         <v>13</v>
       </c>
       <c r="T7" s="22">
-        <v>4823</v>
+        <v>4731</v>
       </c>
       <c r="U7" s="25" t="s">
         <v>135</v>
@@ -4726,7 +4726,7 @@
         <v>13</v>
       </c>
       <c r="T8" s="22">
-        <v>6115</v>
+        <v>4657</v>
       </c>
       <c r="U8" s="25" t="s">
         <v>135</v>
@@ -4797,7 +4797,7 @@
         <v>13</v>
       </c>
       <c r="T9" s="22">
-        <v>4484</v>
+        <v>4603</v>
       </c>
       <c r="U9" s="25" t="s">
         <v>135</v>
@@ -4868,7 +4868,7 @@
         <v>13</v>
       </c>
       <c r="T10" s="22">
-        <v>4992</v>
+        <v>4920</v>
       </c>
       <c r="U10" s="25" t="s">
         <v>135</v>
@@ -4939,7 +4939,7 @@
         <v>13</v>
       </c>
       <c r="T11" s="22">
-        <v>4761</v>
+        <v>5172</v>
       </c>
       <c r="U11" s="25" t="s">
         <v>135</v>
@@ -5010,7 +5010,7 @@
         <v>160</v>
       </c>
       <c r="T12" s="22">
-        <v>4269</v>
+        <v>4829</v>
       </c>
       <c r="U12" s="19" t="s">
         <v>122</v>
@@ -5081,7 +5081,7 @@
         <v>13</v>
       </c>
       <c r="T13" s="22">
-        <v>4093</v>
+        <v>4895</v>
       </c>
       <c r="U13" s="25" t="s">
         <v>135</v>
@@ -5152,7 +5152,7 @@
         <v>13</v>
       </c>
       <c r="T14" s="22">
-        <v>5053</v>
+        <v>5336</v>
       </c>
       <c r="U14" s="25" t="s">
         <v>135</v>
@@ -5223,7 +5223,7 @@
         <v>168</v>
       </c>
       <c r="T15" s="22">
-        <v>5367</v>
+        <v>5861</v>
       </c>
       <c r="U15" s="19" t="s">
         <v>122</v>
@@ -5294,7 +5294,7 @@
         <v>13</v>
       </c>
       <c r="T16" s="22">
-        <v>5619</v>
+        <v>10765</v>
       </c>
       <c r="U16" s="25" t="s">
         <v>135</v>
@@ -5365,7 +5365,7 @@
         <v>13</v>
       </c>
       <c r="T17" s="22">
-        <v>4723</v>
+        <v>5244</v>
       </c>
       <c r="U17" s="25" t="s">
         <v>135</v>
@@ -5436,7 +5436,7 @@
         <v>13</v>
       </c>
       <c r="T18" s="22">
-        <v>5272</v>
+        <v>7146</v>
       </c>
       <c r="U18" s="25" t="s">
         <v>135</v>
@@ -5507,7 +5507,7 @@
         <v>13</v>
       </c>
       <c r="T19" s="22">
-        <v>4750</v>
+        <v>4981</v>
       </c>
       <c r="U19" s="25" t="s">
         <v>135</v>
@@ -5578,7 +5578,7 @@
         <v>13</v>
       </c>
       <c r="T20" s="22">
-        <v>5192</v>
+        <v>4652</v>
       </c>
       <c r="U20" s="25" t="s">
         <v>135</v>
@@ -5649,7 +5649,7 @@
         <v>13</v>
       </c>
       <c r="T21" s="22">
-        <v>4059</v>
+        <v>3297</v>
       </c>
       <c r="U21" s="25" t="s">
         <v>135</v>
@@ -5720,7 +5720,7 @@
         <v>13</v>
       </c>
       <c r="T22" s="22">
-        <v>5006</v>
+        <v>5007</v>
       </c>
       <c r="U22" s="25" t="s">
         <v>135</v>
@@ -5791,7 +5791,7 @@
         <v>13</v>
       </c>
       <c r="T23" s="22">
-        <v>5047</v>
+        <v>4936</v>
       </c>
       <c r="U23" s="25" t="s">
         <v>135</v>
@@ -5862,7 +5862,7 @@
         <v>13</v>
       </c>
       <c r="T24" s="22">
-        <v>4737</v>
+        <v>4925</v>
       </c>
       <c r="U24" s="25" t="s">
         <v>135</v>
@@ -5933,7 +5933,7 @@
         <v>13</v>
       </c>
       <c r="T25" s="22">
-        <v>5268</v>
+        <v>4969</v>
       </c>
       <c r="U25" s="25" t="s">
         <v>135</v>
@@ -6004,7 +6004,7 @@
         <v>13</v>
       </c>
       <c r="T26" s="22">
-        <v>4736</v>
+        <v>5284</v>
       </c>
       <c r="U26" s="25" t="s">
         <v>135</v>
@@ -6075,7 +6075,7 @@
         <v>13</v>
       </c>
       <c r="T27" s="22">
-        <v>6288</v>
+        <v>4558</v>
       </c>
       <c r="U27" s="25" t="s">
         <v>135</v>
@@ -6146,7 +6146,7 @@
         <v>13</v>
       </c>
       <c r="T28" s="22">
-        <v>5312</v>
+        <v>4013</v>
       </c>
       <c r="U28" s="25" t="s">
         <v>135</v>
@@ -6217,7 +6217,7 @@
         <v>200</v>
       </c>
       <c r="T29" s="22">
-        <v>4676</v>
+        <v>4225</v>
       </c>
       <c r="U29" s="19" t="s">
         <v>122</v>
@@ -6288,7 +6288,7 @@
         <v>13</v>
       </c>
       <c r="T30" s="22">
-        <v>5026</v>
+        <v>4971</v>
       </c>
       <c r="U30" s="25" t="s">
         <v>135</v>
@@ -6359,7 +6359,7 @@
         <v>13</v>
       </c>
       <c r="T31" s="22">
-        <v>5767</v>
+        <v>5180</v>
       </c>
       <c r="U31" s="25" t="s">
         <v>135</v>
@@ -6430,7 +6430,7 @@
         <v>13</v>
       </c>
       <c r="T32" s="22">
-        <v>4765</v>
+        <v>4384</v>
       </c>
       <c r="U32" s="25" t="s">
         <v>135</v>
@@ -6501,7 +6501,7 @@
         <v>13</v>
       </c>
       <c r="T33" s="22">
-        <v>6760</v>
+        <v>9626</v>
       </c>
       <c r="U33" s="25" t="s">
         <v>135</v>
@@ -6572,7 +6572,7 @@
         <v>13</v>
       </c>
       <c r="T34" s="22">
-        <v>5188</v>
+        <v>7176</v>
       </c>
       <c r="U34" s="25" t="s">
         <v>135</v>
@@ -6643,7 +6643,7 @@
         <v>13</v>
       </c>
       <c r="T35" s="22">
-        <v>5036</v>
+        <v>5403</v>
       </c>
       <c r="U35" s="25" t="s">
         <v>135</v>
@@ -6714,7 +6714,7 @@
         <v>13</v>
       </c>
       <c r="T36" s="22">
-        <v>4245</v>
+        <v>4067</v>
       </c>
       <c r="U36" s="25" t="s">
         <v>135</v>
@@ -6785,7 +6785,7 @@
         <v>13</v>
       </c>
       <c r="T37" s="22">
-        <v>5210</v>
+        <v>5979</v>
       </c>
       <c r="U37" s="25" t="s">
         <v>135</v>
@@ -6854,7 +6854,7 @@
         <v>13</v>
       </c>
       <c r="T38" s="22">
-        <v>30120</v>
+        <v>30130</v>
       </c>
       <c r="U38" s="25" t="s">
         <v>135</v>
@@ -6925,7 +6925,7 @@
         <v>13</v>
       </c>
       <c r="T39" s="22">
-        <v>5780</v>
+        <v>5241</v>
       </c>
       <c r="U39" s="25" t="s">
         <v>135</v>
@@ -6996,7 +6996,7 @@
         <v>225</v>
       </c>
       <c r="T40" s="22">
-        <v>4289</v>
+        <v>4224</v>
       </c>
       <c r="U40" s="19" t="s">
         <v>122</v>
@@ -7067,7 +7067,7 @@
         <v>229</v>
       </c>
       <c r="T41" s="22">
-        <v>4815</v>
+        <v>4864</v>
       </c>
       <c r="U41" s="19" t="s">
         <v>122</v>
@@ -7138,7 +7138,7 @@
         <v>234</v>
       </c>
       <c r="T42" s="22">
-        <v>5047</v>
+        <v>5642</v>
       </c>
       <c r="U42" s="19" t="s">
         <v>122</v>
@@ -7209,7 +7209,7 @@
         <v>238</v>
       </c>
       <c r="T43" s="22">
-        <v>4630</v>
+        <v>3946</v>
       </c>
       <c r="U43" s="19" t="s">
         <v>122</v>
@@ -7280,7 +7280,7 @@
         <v>242</v>
       </c>
       <c r="T44" s="22">
-        <v>4343</v>
+        <v>4104</v>
       </c>
       <c r="U44" s="19" t="s">
         <v>122</v>
@@ -7351,7 +7351,7 @@
         <v>249</v>
       </c>
       <c r="T45" s="22">
-        <v>3993</v>
+        <v>4143</v>
       </c>
       <c r="U45" s="19" t="s">
         <v>122</v>
@@ -7422,7 +7422,7 @@
         <v>254</v>
       </c>
       <c r="T46" s="22">
-        <v>7378</v>
+        <v>4120</v>
       </c>
       <c r="U46" s="19" t="s">
         <v>122</v>
@@ -7493,7 +7493,7 @@
         <v>259</v>
       </c>
       <c r="T47" s="22">
-        <v>4531</v>
+        <v>4776</v>
       </c>
       <c r="U47" s="19" t="s">
         <v>122</v>
@@ -7564,7 +7564,7 @@
         <v>266</v>
       </c>
       <c r="T48" s="22">
-        <v>4468</v>
+        <v>4201</v>
       </c>
       <c r="U48" s="19" t="s">
         <v>122</v>
@@ -7635,7 +7635,7 @@
         <v>271</v>
       </c>
       <c r="T49" s="22">
-        <v>4643</v>
+        <v>4708</v>
       </c>
       <c r="U49" s="19" t="s">
         <v>122</v>
@@ -7706,7 +7706,7 @@
         <v>13</v>
       </c>
       <c r="T50" s="22">
-        <v>5170</v>
+        <v>5315</v>
       </c>
       <c r="U50" s="25" t="s">
         <v>135</v>
@@ -7753,7 +7753,7 @@
         <v>10</v>
       </c>
       <c r="L51" s="20">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="M51" s="21">
         <v>36</v>
@@ -7777,7 +7777,7 @@
         <v>13</v>
       </c>
       <c r="T51" s="22">
-        <v>17909</v>
+        <v>5849</v>
       </c>
       <c r="U51" s="25" t="s">
         <v>135</v>
@@ -9753,7 +9753,7 @@
         <v>10</v>
       </c>
       <c r="D51">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E51" s="32" t="s">
         <v>282</v>

</xml_diff>

<commit_message>
Sprint 2 CI-012 largest pages complete
</commit_message>
<xml_diff>
--- a/output/ClubHubInsight.xlsx
+++ b/output/ClubHubInsight.xlsx
@@ -19,13 +19,14 @@
     <sheet sheetId="10" name="Media Inventory" state="visible" r:id="rId13"/>
     <sheet sheetId="11" name="Website Composition" state="visible" r:id="rId14"/>
     <sheet sheetId="12" name="Most Referenced" state="visible" r:id="rId15"/>
+    <sheet sheetId="13" name="Largest Pages" state="visible" r:id="rId16"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1570" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1638" uniqueCount="328">
   <si>
     <t>ClubHub Insight</t>
   </si>
@@ -82,13 +83,13 @@
     <t>Crawl Date</t>
   </si>
   <si>
-    <t>02/09/2026, 12:58:34</t>
+    <t>02/09/2026, 16:13:02</t>
   </si>
   <si>
     <t>Crawl Duration</t>
   </si>
   <si>
-    <t>4m 51s</t>
+    <t>5m 2s</t>
   </si>
   <si>
     <t>Version</t>
@@ -139,7 +140,7 @@
     <t>Average Page Load (ms)</t>
   </si>
   <si>
-    <t>5660 ms</t>
+    <t>5850 ms</t>
   </si>
   <si>
     <t>Site Structure</t>
@@ -1004,6 +1005,12 @@
   </si>
   <si>
     <t>Rank</t>
+  </si>
+  <si>
+    <t>HTML Size (Bytes)</t>
+  </si>
+  <si>
+    <t>HTML Size (KB)</t>
   </si>
 </sst>
 </file>
@@ -3625,6 +3632,572 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H21"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="65" customWidth="1"/>
+    <col min="3" max="3" width="75" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="8" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>325</v>
+      </c>
+      <c r="B1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E1" t="s">
+        <v>326</v>
+      </c>
+      <c r="F1" t="s">
+        <v>327</v>
+      </c>
+      <c r="G1" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E2">
+        <v>525642</v>
+      </c>
+      <c r="F2">
+        <v>513.3</v>
+      </c>
+      <c r="G2">
+        <v>25</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>209</v>
+      </c>
+      <c r="C3" t="s">
+        <v>210</v>
+      </c>
+      <c r="D3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E3">
+        <v>487051</v>
+      </c>
+      <c r="F3">
+        <v>475.6</v>
+      </c>
+      <c r="G3">
+        <v>34</v>
+      </c>
+      <c r="H3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>215</v>
+      </c>
+      <c r="C4" t="s">
+        <v>216</v>
+      </c>
+      <c r="D4" t="s">
+        <v>140</v>
+      </c>
+      <c r="E4">
+        <v>484186</v>
+      </c>
+      <c r="F4">
+        <v>472.8</v>
+      </c>
+      <c r="G4">
+        <v>34</v>
+      </c>
+      <c r="H4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>207</v>
+      </c>
+      <c r="C5" t="s">
+        <v>208</v>
+      </c>
+      <c r="D5" t="s">
+        <v>140</v>
+      </c>
+      <c r="E5">
+        <v>483350</v>
+      </c>
+      <c r="F5">
+        <v>472</v>
+      </c>
+      <c r="G5">
+        <v>35</v>
+      </c>
+      <c r="H5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>267</v>
+      </c>
+      <c r="C6" t="s">
+        <v>268</v>
+      </c>
+      <c r="D6" t="s">
+        <v>126</v>
+      </c>
+      <c r="E6">
+        <v>482920</v>
+      </c>
+      <c r="F6">
+        <v>471.6</v>
+      </c>
+      <c r="G6">
+        <v>25</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>219</v>
+      </c>
+      <c r="C7" t="s">
+        <v>220</v>
+      </c>
+      <c r="D7" t="s">
+        <v>140</v>
+      </c>
+      <c r="E7">
+        <v>481949</v>
+      </c>
+      <c r="F7">
+        <v>470.7</v>
+      </c>
+      <c r="G7">
+        <v>33</v>
+      </c>
+      <c r="H7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>137</v>
+      </c>
+      <c r="C8" t="s">
+        <v>138</v>
+      </c>
+      <c r="D8" t="s">
+        <v>140</v>
+      </c>
+      <c r="E8">
+        <v>481315</v>
+      </c>
+      <c r="F8">
+        <v>470</v>
+      </c>
+      <c r="G8">
+        <v>37</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>274</v>
+      </c>
+      <c r="C9" t="s">
+        <v>275</v>
+      </c>
+      <c r="D9" t="s">
+        <v>140</v>
+      </c>
+      <c r="E9">
+        <v>480751</v>
+      </c>
+      <c r="F9">
+        <v>469.5</v>
+      </c>
+      <c r="G9">
+        <v>36</v>
+      </c>
+      <c r="H9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>272</v>
+      </c>
+      <c r="C10" t="s">
+        <v>273</v>
+      </c>
+      <c r="D10" t="s">
+        <v>140</v>
+      </c>
+      <c r="E10">
+        <v>477622</v>
+      </c>
+      <c r="F10">
+        <v>466.4</v>
+      </c>
+      <c r="G10">
+        <v>34</v>
+      </c>
+      <c r="H10">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>131</v>
+      </c>
+      <c r="C11" t="s">
+        <v>132</v>
+      </c>
+      <c r="D11" t="s">
+        <v>133</v>
+      </c>
+      <c r="E11">
+        <v>476699</v>
+      </c>
+      <c r="F11">
+        <v>465.5</v>
+      </c>
+      <c r="G11">
+        <v>29</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>203</v>
+      </c>
+      <c r="C12" t="s">
+        <v>204</v>
+      </c>
+      <c r="D12" t="s">
+        <v>205</v>
+      </c>
+      <c r="E12">
+        <v>461677</v>
+      </c>
+      <c r="F12">
+        <v>450.9</v>
+      </c>
+      <c r="G12">
+        <v>31</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>201</v>
+      </c>
+      <c r="C13" t="s">
+        <v>202</v>
+      </c>
+      <c r="D13" t="s">
+        <v>133</v>
+      </c>
+      <c r="E13">
+        <v>454631</v>
+      </c>
+      <c r="F13">
+        <v>444</v>
+      </c>
+      <c r="G13">
+        <v>25</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>191</v>
+      </c>
+      <c r="C14" t="s">
+        <v>192</v>
+      </c>
+      <c r="D14" t="s">
+        <v>151</v>
+      </c>
+      <c r="E14">
+        <v>439113</v>
+      </c>
+      <c r="F14">
+        <v>428.8</v>
+      </c>
+      <c r="G14">
+        <v>35</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>175</v>
+      </c>
+      <c r="C15" t="s">
+        <v>176</v>
+      </c>
+      <c r="D15" t="s">
+        <v>151</v>
+      </c>
+      <c r="E15">
+        <v>437559</v>
+      </c>
+      <c r="F15">
+        <v>427.3</v>
+      </c>
+      <c r="G15">
+        <v>35</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>189</v>
+      </c>
+      <c r="C16" t="s">
+        <v>190</v>
+      </c>
+      <c r="D16" t="s">
+        <v>151</v>
+      </c>
+      <c r="E16">
+        <v>436130</v>
+      </c>
+      <c r="F16">
+        <v>425.9</v>
+      </c>
+      <c r="G16">
+        <v>35</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>143</v>
+      </c>
+      <c r="C17" t="s">
+        <v>144</v>
+      </c>
+      <c r="D17" t="s">
+        <v>140</v>
+      </c>
+      <c r="E17">
+        <v>435243</v>
+      </c>
+      <c r="F17">
+        <v>425</v>
+      </c>
+      <c r="G17">
+        <v>30</v>
+      </c>
+      <c r="H17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>169</v>
+      </c>
+      <c r="C18" t="s">
+        <v>170</v>
+      </c>
+      <c r="D18" t="s">
+        <v>151</v>
+      </c>
+      <c r="E18">
+        <v>432173</v>
+      </c>
+      <c r="F18">
+        <v>422</v>
+      </c>
+      <c r="G18">
+        <v>34</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>141</v>
+      </c>
+      <c r="C19" t="s">
+        <v>142</v>
+      </c>
+      <c r="D19" t="s">
+        <v>133</v>
+      </c>
+      <c r="E19">
+        <v>431210</v>
+      </c>
+      <c r="F19">
+        <v>421.1</v>
+      </c>
+      <c r="G19">
+        <v>29</v>
+      </c>
+      <c r="H19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>211</v>
+      </c>
+      <c r="C20" t="s">
+        <v>212</v>
+      </c>
+      <c r="D20" t="s">
+        <v>133</v>
+      </c>
+      <c r="E20">
+        <v>430548</v>
+      </c>
+      <c r="F20">
+        <v>420.5</v>
+      </c>
+      <c r="G20">
+        <v>29</v>
+      </c>
+      <c r="H20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>174</v>
+      </c>
+      <c r="C21" t="s">
+        <v>139</v>
+      </c>
+      <c r="D21" t="s">
+        <v>148</v>
+      </c>
+      <c r="E21">
+        <v>415804</v>
+      </c>
+      <c r="F21">
+        <v>406.1</v>
+      </c>
+      <c r="G21">
+        <v>25</v>
+      </c>
+      <c r="H21">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
@@ -4300,7 +4873,7 @@
         <v>121</v>
       </c>
       <c r="T2" s="22">
-        <v>4954</v>
+        <v>4811</v>
       </c>
       <c r="U2" s="19" t="s">
         <v>122</v>
@@ -4371,7 +4944,7 @@
         <v>130</v>
       </c>
       <c r="T3" s="22">
-        <v>3815</v>
+        <v>4820</v>
       </c>
       <c r="U3" s="19" t="s">
         <v>122</v>
@@ -4442,7 +5015,7 @@
         <v>13</v>
       </c>
       <c r="T4" s="22">
-        <v>6357</v>
+        <v>5798</v>
       </c>
       <c r="U4" s="25" t="s">
         <v>135</v>
@@ -4513,7 +5086,7 @@
         <v>13</v>
       </c>
       <c r="T5" s="22">
-        <v>5777</v>
+        <v>6191</v>
       </c>
       <c r="U5" s="25" t="s">
         <v>135</v>
@@ -4584,7 +5157,7 @@
         <v>13</v>
       </c>
       <c r="T6" s="22">
-        <v>5061</v>
+        <v>5919</v>
       </c>
       <c r="U6" s="25" t="s">
         <v>135</v>
@@ -4655,7 +5228,7 @@
         <v>13</v>
       </c>
       <c r="T7" s="22">
-        <v>4731</v>
+        <v>5114</v>
       </c>
       <c r="U7" s="25" t="s">
         <v>135</v>
@@ -4726,7 +5299,7 @@
         <v>13</v>
       </c>
       <c r="T8" s="22">
-        <v>4657</v>
+        <v>5129</v>
       </c>
       <c r="U8" s="25" t="s">
         <v>135</v>
@@ -4797,7 +5370,7 @@
         <v>13</v>
       </c>
       <c r="T9" s="22">
-        <v>4603</v>
+        <v>4842</v>
       </c>
       <c r="U9" s="25" t="s">
         <v>135</v>
@@ -4868,7 +5441,7 @@
         <v>13</v>
       </c>
       <c r="T10" s="22">
-        <v>4920</v>
+        <v>4700</v>
       </c>
       <c r="U10" s="25" t="s">
         <v>135</v>
@@ -4939,7 +5512,7 @@
         <v>13</v>
       </c>
       <c r="T11" s="22">
-        <v>5172</v>
+        <v>6629</v>
       </c>
       <c r="U11" s="25" t="s">
         <v>135</v>
@@ -5010,7 +5583,7 @@
         <v>160</v>
       </c>
       <c r="T12" s="22">
-        <v>4829</v>
+        <v>4921</v>
       </c>
       <c r="U12" s="19" t="s">
         <v>122</v>
@@ -5081,7 +5654,7 @@
         <v>13</v>
       </c>
       <c r="T13" s="22">
-        <v>4895</v>
+        <v>4338</v>
       </c>
       <c r="U13" s="25" t="s">
         <v>135</v>
@@ -5152,7 +5725,7 @@
         <v>13</v>
       </c>
       <c r="T14" s="22">
-        <v>5336</v>
+        <v>5363</v>
       </c>
       <c r="U14" s="25" t="s">
         <v>135</v>
@@ -5223,7 +5796,7 @@
         <v>168</v>
       </c>
       <c r="T15" s="22">
-        <v>5861</v>
+        <v>5259</v>
       </c>
       <c r="U15" s="19" t="s">
         <v>122</v>
@@ -5294,7 +5867,7 @@
         <v>13</v>
       </c>
       <c r="T16" s="22">
-        <v>10765</v>
+        <v>5116</v>
       </c>
       <c r="U16" s="25" t="s">
         <v>135</v>
@@ -5365,7 +5938,7 @@
         <v>13</v>
       </c>
       <c r="T17" s="22">
-        <v>5244</v>
+        <v>4628</v>
       </c>
       <c r="U17" s="25" t="s">
         <v>135</v>
@@ -5436,7 +6009,7 @@
         <v>13</v>
       </c>
       <c r="T18" s="22">
-        <v>7146</v>
+        <v>6062</v>
       </c>
       <c r="U18" s="25" t="s">
         <v>135</v>
@@ -5507,7 +6080,7 @@
         <v>13</v>
       </c>
       <c r="T19" s="22">
-        <v>4981</v>
+        <v>5377</v>
       </c>
       <c r="U19" s="25" t="s">
         <v>135</v>
@@ -5578,7 +6151,7 @@
         <v>13</v>
       </c>
       <c r="T20" s="22">
-        <v>4652</v>
+        <v>4982</v>
       </c>
       <c r="U20" s="25" t="s">
         <v>135</v>
@@ -5649,7 +6222,7 @@
         <v>13</v>
       </c>
       <c r="T21" s="22">
-        <v>3297</v>
+        <v>3504</v>
       </c>
       <c r="U21" s="25" t="s">
         <v>135</v>
@@ -5720,7 +6293,7 @@
         <v>13</v>
       </c>
       <c r="T22" s="22">
-        <v>5007</v>
+        <v>5204</v>
       </c>
       <c r="U22" s="25" t="s">
         <v>135</v>
@@ -5791,7 +6364,7 @@
         <v>13</v>
       </c>
       <c r="T23" s="22">
-        <v>4936</v>
+        <v>7001</v>
       </c>
       <c r="U23" s="25" t="s">
         <v>135</v>
@@ -5862,7 +6435,7 @@
         <v>13</v>
       </c>
       <c r="T24" s="22">
-        <v>4925</v>
+        <v>6399</v>
       </c>
       <c r="U24" s="25" t="s">
         <v>135</v>
@@ -5933,7 +6506,7 @@
         <v>13</v>
       </c>
       <c r="T25" s="22">
-        <v>4969</v>
+        <v>5758</v>
       </c>
       <c r="U25" s="25" t="s">
         <v>135</v>
@@ -6004,7 +6577,7 @@
         <v>13</v>
       </c>
       <c r="T26" s="22">
-        <v>5284</v>
+        <v>5741</v>
       </c>
       <c r="U26" s="25" t="s">
         <v>135</v>
@@ -6075,7 +6648,7 @@
         <v>13</v>
       </c>
       <c r="T27" s="22">
-        <v>4558</v>
+        <v>5093</v>
       </c>
       <c r="U27" s="25" t="s">
         <v>135</v>
@@ -6146,7 +6719,7 @@
         <v>13</v>
       </c>
       <c r="T28" s="22">
-        <v>4013</v>
+        <v>4945</v>
       </c>
       <c r="U28" s="25" t="s">
         <v>135</v>
@@ -6217,7 +6790,7 @@
         <v>200</v>
       </c>
       <c r="T29" s="22">
-        <v>4225</v>
+        <v>5421</v>
       </c>
       <c r="U29" s="19" t="s">
         <v>122</v>
@@ -6288,7 +6861,7 @@
         <v>13</v>
       </c>
       <c r="T30" s="22">
-        <v>4971</v>
+        <v>4838</v>
       </c>
       <c r="U30" s="25" t="s">
         <v>135</v>
@@ -6359,7 +6932,7 @@
         <v>13</v>
       </c>
       <c r="T31" s="22">
-        <v>5180</v>
+        <v>5610</v>
       </c>
       <c r="U31" s="25" t="s">
         <v>135</v>
@@ -6430,7 +7003,7 @@
         <v>13</v>
       </c>
       <c r="T32" s="22">
-        <v>4384</v>
+        <v>4746</v>
       </c>
       <c r="U32" s="25" t="s">
         <v>135</v>
@@ -6501,7 +7074,7 @@
         <v>13</v>
       </c>
       <c r="T33" s="22">
-        <v>9626</v>
+        <v>6125</v>
       </c>
       <c r="U33" s="25" t="s">
         <v>135</v>
@@ -6572,7 +7145,7 @@
         <v>13</v>
       </c>
       <c r="T34" s="22">
-        <v>7176</v>
+        <v>6220</v>
       </c>
       <c r="U34" s="25" t="s">
         <v>135</v>
@@ -6643,7 +7216,7 @@
         <v>13</v>
       </c>
       <c r="T35" s="22">
-        <v>5403</v>
+        <v>5228</v>
       </c>
       <c r="U35" s="25" t="s">
         <v>135</v>
@@ -6714,7 +7287,7 @@
         <v>13</v>
       </c>
       <c r="T36" s="22">
-        <v>4067</v>
+        <v>4264</v>
       </c>
       <c r="U36" s="25" t="s">
         <v>135</v>
@@ -6785,7 +7358,7 @@
         <v>13</v>
       </c>
       <c r="T37" s="22">
-        <v>5979</v>
+        <v>5772</v>
       </c>
       <c r="U37" s="25" t="s">
         <v>135</v>
@@ -6854,7 +7427,7 @@
         <v>13</v>
       </c>
       <c r="T38" s="22">
-        <v>30130</v>
+        <v>30116</v>
       </c>
       <c r="U38" s="25" t="s">
         <v>135</v>
@@ -6925,7 +7498,7 @@
         <v>13</v>
       </c>
       <c r="T39" s="22">
-        <v>5241</v>
+        <v>6106</v>
       </c>
       <c r="U39" s="25" t="s">
         <v>135</v>
@@ -6996,7 +7569,7 @@
         <v>225</v>
       </c>
       <c r="T40" s="22">
-        <v>4224</v>
+        <v>5846</v>
       </c>
       <c r="U40" s="19" t="s">
         <v>122</v>
@@ -7067,7 +7640,7 @@
         <v>229</v>
       </c>
       <c r="T41" s="22">
-        <v>4864</v>
+        <v>4952</v>
       </c>
       <c r="U41" s="19" t="s">
         <v>122</v>
@@ -7138,7 +7711,7 @@
         <v>234</v>
       </c>
       <c r="T42" s="22">
-        <v>5642</v>
+        <v>5397</v>
       </c>
       <c r="U42" s="19" t="s">
         <v>122</v>
@@ -7209,7 +7782,7 @@
         <v>238</v>
       </c>
       <c r="T43" s="22">
-        <v>3946</v>
+        <v>4615</v>
       </c>
       <c r="U43" s="19" t="s">
         <v>122</v>
@@ -7280,7 +7853,7 @@
         <v>242</v>
       </c>
       <c r="T44" s="22">
-        <v>4104</v>
+        <v>4894</v>
       </c>
       <c r="U44" s="19" t="s">
         <v>122</v>
@@ -7351,7 +7924,7 @@
         <v>249</v>
       </c>
       <c r="T45" s="22">
-        <v>4143</v>
+        <v>5923</v>
       </c>
       <c r="U45" s="19" t="s">
         <v>122</v>
@@ -7422,7 +7995,7 @@
         <v>254</v>
       </c>
       <c r="T46" s="22">
-        <v>4120</v>
+        <v>5203</v>
       </c>
       <c r="U46" s="19" t="s">
         <v>122</v>
@@ -7493,7 +8066,7 @@
         <v>259</v>
       </c>
       <c r="T47" s="22">
-        <v>4776</v>
+        <v>3981</v>
       </c>
       <c r="U47" s="19" t="s">
         <v>122</v>
@@ -7564,7 +8137,7 @@
         <v>266</v>
       </c>
       <c r="T48" s="22">
-        <v>4201</v>
+        <v>4814</v>
       </c>
       <c r="U48" s="19" t="s">
         <v>122</v>
@@ -7635,7 +8208,7 @@
         <v>271</v>
       </c>
       <c r="T49" s="22">
-        <v>4708</v>
+        <v>6621</v>
       </c>
       <c r="U49" s="19" t="s">
         <v>122</v>
@@ -7706,7 +8279,7 @@
         <v>13</v>
       </c>
       <c r="T50" s="22">
-        <v>5315</v>
+        <v>6468</v>
       </c>
       <c r="U50" s="25" t="s">
         <v>135</v>
@@ -7777,7 +8350,7 @@
         <v>13</v>
       </c>
       <c r="T51" s="22">
-        <v>5849</v>
+        <v>5719</v>
       </c>
       <c r="U51" s="25" t="s">
         <v>135</v>

</xml_diff>